<commit_message>
Comentarios mejorados, las imágenes se suben de una vez
</commit_message>
<xml_diff>
--- a/data/DatosFirestore.xlsx
+++ b/data/DatosFirestore.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DAM\Proyecto Final\Nueva carpeta\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B32F1AC1-6ABE-4534-B439-6906FACF54D8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27CC034A-74A6-4CBC-B2DC-B5660318597F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" xr2:uid="{F7709132-0D59-47A5-B484-42C89F632E94}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="345">
   <si>
     <t>Nombre</t>
   </si>
@@ -115,9 +115,6 @@
     <t>l</t>
   </si>
   <si>
-    <t>u</t>
-  </si>
-  <si>
     <t>cl</t>
   </si>
   <si>
@@ -622,9 +619,6 @@
     <t>Congelados</t>
   </si>
   <si>
-    <t>Pizzas y platos preparados</t>
-  </si>
-  <si>
     <t>Guisantes congelados Findus</t>
   </si>
   <si>
@@ -977,6 +971,96 @@
   </si>
   <si>
     <t>alpeso</t>
+  </si>
+  <si>
+    <t>Ketchup Orlando</t>
+  </si>
+  <si>
+    <t>Salsa de tomate ketchup, ideal para acompañar hamburguesas, perritos calientes y patatas fritas. Envase de 300 g.</t>
+  </si>
+  <si>
+    <t>Cervezas</t>
+  </si>
+  <si>
+    <t>Lata de Aquarius Melocotón Rojo</t>
+  </si>
+  <si>
+    <t>Bebida refrescante aromatizada con sales minerales, sabor melocotón rojo. Fuente de zinc y selenio. Lata de 33 cl.</t>
+  </si>
+  <si>
+    <t>Canelones El Pavo</t>
+  </si>
+  <si>
+    <t>Platos preparados</t>
+  </si>
+  <si>
+    <t>Amstel Oro 0,0 Tostada</t>
+  </si>
+  <si>
+    <t>Cerveza sin alcohol tipo Lager, con un sabor intenso a malta tostada y un amargor equilibrado. Lata de 33 cl.</t>
+  </si>
+  <si>
+    <t>Fanta de Naranja Zero Azúcares</t>
+  </si>
+  <si>
+    <t>Refresco de naranja sin azúcares añadidos y con el sabor original de Fanta. Lata de 33 cl.</t>
+  </si>
+  <si>
+    <t>ketchuporlandobarrilito300gr.png</t>
+  </si>
+  <si>
+    <t>cervezaamsteloro00tostadalata33cl.png</t>
+  </si>
+  <si>
+    <t>can_redpeach.png</t>
+  </si>
+  <si>
+    <t>ZumoTropical.png</t>
+  </si>
+  <si>
+    <t>Zumo Tropical Hacendado</t>
+  </si>
+  <si>
+    <t>ud</t>
+  </si>
+  <si>
+    <t>Gluten. Huevo, Soja, Mostaza</t>
+  </si>
+  <si>
+    <t>Zumo de frutas tropicales (uva, piña, mango y manzana) con leche sin azúcares añadidos. Pack de 6 zumos de 200 ml.</t>
+  </si>
+  <si>
+    <t>Canelones-El-Pavo.png</t>
+  </si>
+  <si>
+    <t>Placas precocidas para canelones. Las auténticas placas tradicionales El Pavo, elaboradas siguiendo el mismo proceso tradicional desde hace más de 120 años. Elaboradas con una cuidada selección de harinas de trigo blando, dándole un grosor y textura únicos, garantizando un dente perfecto. Envase de 20 placas, 120 g.</t>
+  </si>
+  <si>
+    <t>FantaZero.png</t>
+  </si>
+  <si>
+    <t>Almendras tostadas ligeramente saladas, perfectas como aperitivo o para ensaladas. Bolsa de 200 g.</t>
+  </si>
+  <si>
+    <t>Frutos secos</t>
+  </si>
+  <si>
+    <t>Almendras</t>
+  </si>
+  <si>
+    <t>coosol.png</t>
+  </si>
+  <si>
+    <t>Aceite de girasol especial freír Coosol</t>
+  </si>
+  <si>
+    <t>Aceite de girasol alto oleico, ideal para freír. Garrafa de 5 litros.</t>
+  </si>
+  <si>
+    <t>Almendras tostadas Frit Ravich</t>
+  </si>
+  <si>
+    <t>almendras.png</t>
   </si>
 </sst>
 </file>
@@ -1704,16 +1788,16 @@
         <v>26</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N1" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="O1" s="40" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="30" x14ac:dyDescent="0.25">
@@ -1733,22 +1817,22 @@
         <v>8</v>
       </c>
       <c r="F2" s="33">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="G2" s="34" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="H2" s="33">
         <v>123</v>
       </c>
       <c r="I2" s="35" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J2" s="36">
         <v>33</v>
       </c>
       <c r="K2" s="35" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="L2" s="37"/>
       <c r="M2" s="35"/>
@@ -1776,19 +1860,19 @@
         <v>200</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="H3" s="5">
         <v>1234</v>
       </c>
       <c r="I3" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J3" s="9">
         <v>33</v>
       </c>
       <c r="K3" s="10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="L3" s="12"/>
       <c r="M3" s="10"/>
@@ -1816,7 +1900,7 @@
         <v>30</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="H4" s="5">
         <v>12345</v>
@@ -1826,7 +1910,7 @@
         <v>1</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>29</v>
+        <v>331</v>
       </c>
       <c r="L4" s="12"/>
       <c r="M4" s="10"/>
@@ -1836,7 +1920,7 @@
     </row>
     <row r="5" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="28" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>20</v>
@@ -1854,7 +1938,7 @@
         <v>250</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="H5" s="5">
         <v>8431876267259</v>
@@ -1883,7 +1967,7 @@
         <v>5.7</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>21</v>
@@ -1892,13 +1976,13 @@
         <v>67</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="H6" s="5">
         <v>333</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="J6" s="9">
         <v>1455</v>
@@ -1908,7 +1992,7 @@
       </c>
       <c r="L6" s="12"/>
       <c r="M6" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="N6" s="26">
         <v>10</v>
@@ -1916,25 +2000,25 @@
     </row>
     <row r="7" spans="1:15" ht="135" x14ac:dyDescent="0.25">
       <c r="A7" s="28" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C7" s="3">
         <v>1.95</v>
       </c>
       <c r="D7" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" s="11" t="s">
         <v>34</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>35</v>
       </c>
       <c r="F7" s="5">
         <v>30</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="H7" s="5">
         <v>999</v>
@@ -1944,11 +2028,11 @@
         <v>1</v>
       </c>
       <c r="K7" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L7" s="13"/>
       <c r="M7" s="25" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="N7" s="26">
         <v>4</v>
@@ -1956,25 +2040,25 @@
     </row>
     <row r="8" spans="1:15" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>38</v>
       </c>
       <c r="C8" s="3">
         <v>1.99</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F8" s="5">
         <v>100</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="H8" s="5">
         <v>998</v>
@@ -1984,7 +2068,7 @@
         <v>75</v>
       </c>
       <c r="K8" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L8" s="12"/>
       <c r="M8" s="10"/>
@@ -1994,25 +2078,25 @@
     </row>
     <row r="9" spans="1:15" ht="75" x14ac:dyDescent="0.25">
       <c r="A9" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>41</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>42</v>
       </c>
       <c r="C9" s="3">
         <v>1.65</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F9" s="5">
         <v>240</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H9" s="5">
         <v>997</v>
@@ -2022,11 +2106,11 @@
         <v>200</v>
       </c>
       <c r="K9" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L9" s="12"/>
       <c r="M9" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N9" s="26">
         <v>4</v>
@@ -2034,25 +2118,25 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="28" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C10" s="3">
         <v>1.88</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F10" s="5">
         <v>76</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H10" s="5">
         <v>996</v>
@@ -2062,7 +2146,7 @@
         <v>1</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L10" s="12"/>
       <c r="M10" s="10"/>
@@ -2072,25 +2156,25 @@
     </row>
     <row r="11" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="28" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C11" s="3">
         <v>6</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="F11" s="5">
         <v>40</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="H11" s="5">
         <v>11111</v>
@@ -2100,7 +2184,7 @@
         <v>1</v>
       </c>
       <c r="K11" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L11" s="12"/>
       <c r="M11" s="10"/>
@@ -2108,30 +2192,30 @@
         <v>4</v>
       </c>
       <c r="O11" s="10" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="12" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="28" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C12" s="3">
         <v>3</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="F12" s="5">
         <v>35</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H12" s="5">
         <v>22222</v>
@@ -2141,7 +2225,7 @@
         <v>1</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L12" s="12"/>
       <c r="M12" s="10"/>
@@ -2149,30 +2233,30 @@
         <v>4</v>
       </c>
       <c r="O12" s="10" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="13" spans="1:15" ht="60" x14ac:dyDescent="0.25">
       <c r="A13" s="28" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C13" s="3">
         <v>1.46</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F13" s="5">
         <v>100</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H13" s="5">
         <v>8431876268584</v>
@@ -2186,7 +2270,7 @@
       </c>
       <c r="L13" s="12"/>
       <c r="M13" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N13" s="26">
         <v>4</v>
@@ -2194,25 +2278,25 @@
     </row>
     <row r="14" spans="1:15" ht="165" x14ac:dyDescent="0.25">
       <c r="A14" s="28" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C14" s="3">
         <v>1.29</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F14" s="5">
         <v>100</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H14" s="5">
         <v>125</v>
@@ -2226,7 +2310,7 @@
       </c>
       <c r="L14" s="12"/>
       <c r="M14" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N14" s="26">
         <v>4</v>
@@ -2234,25 +2318,25 @@
     </row>
     <row r="15" spans="1:15" ht="75" x14ac:dyDescent="0.25">
       <c r="A15" s="28" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C15" s="3">
         <v>2.2999999999999998</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F15" s="5">
         <v>20</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H15" s="5">
         <v>126</v>
@@ -2266,7 +2350,7 @@
       </c>
       <c r="L15" s="12"/>
       <c r="M15" s="10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="N15" s="26">
         <v>10</v>
@@ -2274,25 +2358,25 @@
     </row>
     <row r="16" spans="1:15" ht="60" x14ac:dyDescent="0.25">
       <c r="A16" s="28" t="s">
+        <v>96</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>98</v>
       </c>
       <c r="C16" s="3">
         <v>1.33</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F16" s="5">
         <v>37</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H16" s="5">
         <v>127</v>
@@ -2306,7 +2390,7 @@
       </c>
       <c r="L16" s="12"/>
       <c r="M16" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N16" s="26">
         <v>4</v>
@@ -2314,10 +2398,10 @@
     </row>
     <row r="17" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="28" t="s">
+        <v>100</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>102</v>
       </c>
       <c r="C17" s="3">
         <v>0.5</v>
@@ -2332,7 +2416,7 @@
         <v>150</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="H17" s="5">
         <v>8410123456789</v>
@@ -2342,7 +2426,7 @@
         <v>33</v>
       </c>
       <c r="K17" s="10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="L17" s="12"/>
       <c r="M17" s="10"/>
@@ -2352,10 +2436,10 @@
     </row>
     <row r="18" spans="1:15" ht="60" x14ac:dyDescent="0.25">
       <c r="A18" s="28" t="s">
+        <v>102</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="C18" s="3">
         <v>1.49</v>
@@ -2364,13 +2448,13 @@
         <v>7</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F18" s="5">
         <v>80</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="H18" s="5">
         <v>8410123456790</v>
@@ -2390,10 +2474,10 @@
     </row>
     <row r="19" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="28" t="s">
+        <v>105</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>107</v>
       </c>
       <c r="C19" s="3">
         <v>2.4900000000000002</v>
@@ -2402,13 +2486,13 @@
         <v>7</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F19" s="5">
         <v>40</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="H19" s="5">
         <v>8410123456800</v>
@@ -2428,25 +2512,25 @@
     </row>
     <row r="20" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="28" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C20" s="3">
         <v>1.85</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F20" s="5">
         <v>50</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="H20" s="5">
         <v>8410123456817</v>
@@ -2456,11 +2540,11 @@
         <v>460</v>
       </c>
       <c r="K20" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L20" s="12"/>
       <c r="M20" s="10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="N20" s="26">
         <v>4</v>
@@ -2468,25 +2552,25 @@
     </row>
     <row r="21" spans="1:15" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" s="28" t="s">
+        <v>111</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>113</v>
       </c>
       <c r="C21" s="3">
         <v>2.25</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F21" s="5">
         <v>60</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="H21" s="5">
         <v>8410123456824</v>
@@ -2496,11 +2580,11 @@
         <v>400</v>
       </c>
       <c r="K21" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L21" s="12"/>
       <c r="M21" s="10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="N21" s="26">
         <v>10</v>
@@ -2508,25 +2592,25 @@
     </row>
     <row r="22" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="29" t="s">
+        <v>114</v>
+      </c>
+      <c r="B22" s="39" t="s">
         <v>115</v>
-      </c>
-      <c r="B22" s="39" t="s">
-        <v>116</v>
       </c>
       <c r="C22" s="3">
         <v>1.35</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F22" s="5">
         <v>90</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="H22" s="5">
         <v>8410123456831</v>
@@ -2536,11 +2620,11 @@
         <v>450</v>
       </c>
       <c r="K22" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L22" s="12"/>
       <c r="M22" s="25" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="N22" s="26">
         <v>10</v>
@@ -2548,25 +2632,25 @@
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="29" t="s">
+        <v>117</v>
+      </c>
+      <c r="B23" s="39" t="s">
         <v>118</v>
-      </c>
-      <c r="B23" s="39" t="s">
-        <v>119</v>
       </c>
       <c r="C23" s="3">
         <v>1.65</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F23" s="5">
         <v>70</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="H23" s="5">
         <v>8410123456848</v>
@@ -2576,7 +2660,7 @@
         <v>350</v>
       </c>
       <c r="K23" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L23" s="12"/>
       <c r="M23" s="10"/>
@@ -2586,25 +2670,25 @@
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="29" t="s">
+        <v>120</v>
+      </c>
+      <c r="B24" s="39" t="s">
         <v>121</v>
-      </c>
-      <c r="B24" s="39" t="s">
-        <v>122</v>
       </c>
       <c r="C24" s="3">
         <v>2.95</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F24" s="5">
         <v>120</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="H24" s="5">
         <v>8410123456855</v>
@@ -2614,11 +2698,11 @@
         <v>80</v>
       </c>
       <c r="K24" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L24" s="12"/>
       <c r="M24" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="N24" s="26">
         <v>10</v>
@@ -2626,25 +2710,25 @@
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="29" t="s">
+        <v>123</v>
+      </c>
+      <c r="B25" s="39" t="s">
         <v>124</v>
-      </c>
-      <c r="B25" s="39" t="s">
-        <v>125</v>
       </c>
       <c r="C25" s="3">
         <v>2.29</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F25" s="5">
         <v>85</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="H25" s="5">
         <v>8410123456862</v>
@@ -2654,11 +2738,11 @@
         <v>500</v>
       </c>
       <c r="K25" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L25" s="12"/>
       <c r="M25" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N25" s="26">
         <v>4</v>
@@ -2666,25 +2750,25 @@
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="29" t="s">
+        <v>126</v>
+      </c>
+      <c r="B26" s="39" t="s">
         <v>127</v>
-      </c>
-      <c r="B26" s="39" t="s">
-        <v>128</v>
       </c>
       <c r="C26" s="3">
         <v>2.15</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F26" s="5">
         <v>55</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="H26" s="5">
         <v>8410123456879</v>
@@ -2694,11 +2778,11 @@
         <v>200</v>
       </c>
       <c r="K26" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L26" s="12"/>
       <c r="M26" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N26" s="26">
         <v>4</v>
@@ -2706,25 +2790,25 @@
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="29" t="s">
+        <v>128</v>
+      </c>
+      <c r="B27" s="39" t="s">
         <v>129</v>
-      </c>
-      <c r="B27" s="39" t="s">
-        <v>130</v>
       </c>
       <c r="C27" s="3">
         <v>3.1</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F27" s="5">
         <v>45</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="H27" s="5">
         <v>8410123456886</v>
@@ -2734,7 +2818,7 @@
         <v>340</v>
       </c>
       <c r="K27" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L27" s="12"/>
       <c r="M27" s="10"/>
@@ -2744,25 +2828,25 @@
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="29" t="s">
+        <v>131</v>
+      </c>
+      <c r="B28" s="39" t="s">
         <v>132</v>
-      </c>
-      <c r="B28" s="39" t="s">
-        <v>133</v>
       </c>
       <c r="C28" s="3">
         <v>2.75</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F28" s="5">
         <v>60</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="H28" s="5">
         <v>8410123456893</v>
@@ -2772,7 +2856,7 @@
         <v>350</v>
       </c>
       <c r="K28" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L28" s="12"/>
       <c r="M28" s="10"/>
@@ -2782,10 +2866,10 @@
     </row>
     <row r="29" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="29" t="s">
+        <v>133</v>
+      </c>
+      <c r="B29" s="39" t="s">
         <v>134</v>
-      </c>
-      <c r="B29" s="39" t="s">
-        <v>135</v>
       </c>
       <c r="C29" s="3">
         <v>2.99</v>
@@ -2794,13 +2878,13 @@
         <v>22</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F29" s="5">
         <v>100</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="H29" s="5">
         <v>8410123456909</v>
@@ -2810,11 +2894,11 @@
         <v>150</v>
       </c>
       <c r="K29" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L29" s="12"/>
       <c r="M29" s="25" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="N29" s="26">
         <v>21</v>
@@ -2822,25 +2906,25 @@
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="29" t="s">
+        <v>137</v>
+      </c>
+      <c r="B30" s="39" t="s">
         <v>138</v>
-      </c>
-      <c r="B30" s="39" t="s">
-        <v>139</v>
       </c>
       <c r="C30" s="3">
         <v>2.4900000000000002</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F30" s="5">
         <v>200</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="H30" s="5">
         <v>8410123456916</v>
@@ -2850,11 +2934,11 @@
         <v>300</v>
       </c>
       <c r="K30" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L30" s="12"/>
       <c r="M30" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="N30" s="26">
         <v>4</v>
@@ -2862,25 +2946,25 @@
     </row>
     <row r="31" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="29" t="s">
+        <v>141</v>
+      </c>
+      <c r="B31" s="39" t="s">
         <v>142</v>
-      </c>
-      <c r="B31" s="39" t="s">
-        <v>143</v>
       </c>
       <c r="C31" s="3">
         <v>2.69</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="F31" s="5">
         <v>80</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="H31" s="5">
         <v>33333</v>
@@ -2890,7 +2974,7 @@
         <v>1</v>
       </c>
       <c r="K31" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L31" s="12"/>
       <c r="M31" s="10"/>
@@ -2898,30 +2982,30 @@
         <v>4</v>
       </c>
       <c r="O31" s="10" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="32" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="29" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B32" s="39" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C32" s="3">
         <v>2.39</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="F32" s="5">
         <v>65</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="H32" s="5">
         <v>44444</v>
@@ -2931,7 +3015,7 @@
         <v>1</v>
       </c>
       <c r="K32" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L32" s="12"/>
       <c r="M32" s="10"/>
@@ -2939,30 +3023,30 @@
         <v>4</v>
       </c>
       <c r="O32" s="10" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="33" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="29" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B33" s="39" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C33" s="3">
         <v>2.99</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="F33" s="5">
         <v>50</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="H33" s="5">
         <v>55555</v>
@@ -2972,7 +3056,7 @@
         <v>1</v>
       </c>
       <c r="K33" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L33" s="12"/>
       <c r="M33" s="10"/>
@@ -2980,30 +3064,30 @@
         <v>4</v>
       </c>
       <c r="O33" s="10" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="29" t="s">
+        <v>144</v>
+      </c>
+      <c r="B34" s="39" t="s">
         <v>145</v>
-      </c>
-      <c r="B34" s="39" t="s">
-        <v>146</v>
       </c>
       <c r="C34" s="3">
         <v>6.95</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F34" s="5">
         <v>40</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="H34" s="5">
         <v>8410123456954</v>
@@ -3023,25 +3107,25 @@
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="29" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B35" s="39" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C35" s="3">
         <v>2.25</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F35" s="5">
         <v>35</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="H35" s="5">
         <v>8410123456961</v>
@@ -3061,25 +3145,25 @@
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="29" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B36" s="39" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C36" s="3">
         <v>0.55000000000000004</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F36" s="5">
         <v>150</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="H36" s="5">
         <v>8410123456978</v>
@@ -3089,7 +3173,7 @@
         <v>1</v>
       </c>
       <c r="K36" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L36" s="12"/>
       <c r="M36" s="10"/>
@@ -3099,25 +3183,25 @@
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="29" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B37" s="39" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C37" s="3">
         <v>1.1499999999999999</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F37" s="5">
         <v>120</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H37" s="5">
         <v>8410123456985</v>
@@ -3127,7 +3211,7 @@
         <v>750</v>
       </c>
       <c r="K37" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L37" s="12"/>
       <c r="M37" s="10"/>
@@ -3137,25 +3221,25 @@
     </row>
     <row r="38" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="29" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B38" s="39" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C38" s="3">
         <v>2.99</v>
       </c>
       <c r="D38" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F38" s="5">
         <v>45</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="H38" s="5">
         <v>99999</v>
@@ -3165,7 +3249,7 @@
         <v>1</v>
       </c>
       <c r="K38" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L38" s="12"/>
       <c r="M38" s="10"/>
@@ -3173,30 +3257,30 @@
         <v>4</v>
       </c>
       <c r="O38" s="10" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="29" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B39" s="39" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C39" s="3">
         <v>5.49</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F39" s="5">
         <v>30</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H39" s="5">
         <v>8410123457004</v>
@@ -3206,7 +3290,7 @@
         <v>400</v>
       </c>
       <c r="K39" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L39" s="12"/>
       <c r="M39" s="10"/>
@@ -3216,25 +3300,25 @@
     </row>
     <row r="40" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="29" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B40" s="39" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C40" s="3">
         <v>7.95</v>
       </c>
       <c r="D40" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="E40" s="11" t="s">
         <v>165</v>
-      </c>
-      <c r="E40" s="11" t="s">
-        <v>166</v>
       </c>
       <c r="F40" s="5">
         <v>25</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="H40" s="5">
         <v>8410123457011</v>
@@ -3244,11 +3328,11 @@
         <v>250</v>
       </c>
       <c r="K40" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L40" s="12"/>
       <c r="M40" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="N40" s="26">
         <v>10</v>
@@ -3256,25 +3340,25 @@
     </row>
     <row r="41" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="29" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B41" s="39" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C41" s="3">
         <v>2.75</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F41" s="5">
         <v>60</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="H41" s="5">
         <v>8410123457028</v>
@@ -3284,11 +3368,11 @@
         <v>250</v>
       </c>
       <c r="K41" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L41" s="12"/>
       <c r="M41" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N41" s="26">
         <v>4</v>
@@ -3296,25 +3380,25 @@
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="29" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B42" s="39" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C42" s="3">
         <v>1</v>
       </c>
       <c r="D42" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="E42" s="11" t="s">
         <v>158</v>
-      </c>
-      <c r="E42" s="11" t="s">
-        <v>159</v>
       </c>
       <c r="F42" s="5">
         <v>90</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="H42" s="5">
         <v>8410123457035</v>
@@ -3324,11 +3408,11 @@
         <v>35</v>
       </c>
       <c r="K42" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L42" s="12"/>
       <c r="M42" s="10" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="N42" s="26">
         <v>10</v>
@@ -3336,25 +3420,25 @@
     </row>
     <row r="43" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="29" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B43" s="39" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C43" s="3">
         <v>2.0499999999999998</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F43" s="5">
         <v>55</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="H43" s="5">
         <v>8410123457042</v>
@@ -3364,7 +3448,7 @@
         <v>25</v>
       </c>
       <c r="K43" s="10" t="s">
-        <v>29</v>
+        <v>331</v>
       </c>
       <c r="L43" s="12"/>
       <c r="M43" s="10"/>
@@ -3374,25 +3458,25 @@
     </row>
     <row r="44" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="29" t="s">
+        <v>166</v>
+      </c>
+      <c r="B44" s="39" t="s">
         <v>167</v>
-      </c>
-      <c r="B44" s="39" t="s">
-        <v>168</v>
       </c>
       <c r="C44" s="3">
         <v>2.25</v>
       </c>
       <c r="D44" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E44" s="11" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="F44" s="5">
         <v>70</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="H44" s="5">
         <v>8410123457059</v>
@@ -3402,7 +3486,7 @@
         <v>500</v>
       </c>
       <c r="K44" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L44" s="12"/>
       <c r="M44" s="10"/>
@@ -3412,25 +3496,25 @@
     </row>
     <row r="45" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="29" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B45" s="39" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C45" s="3">
         <v>4.99</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="F45" s="5">
         <v>90</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="H45" s="5">
         <v>66666</v>
@@ -3440,7 +3524,7 @@
         <v>1</v>
       </c>
       <c r="K45" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L45" s="12"/>
       <c r="M45" s="10"/>
@@ -3448,30 +3532,30 @@
         <v>4</v>
       </c>
       <c r="O45" s="10" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="46" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="29" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B46" s="39" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C46" s="3">
         <v>2.42</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E46" s="11" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F46" s="5">
         <v>55</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="H46" s="5">
         <v>77777</v>
@@ -3481,7 +3565,7 @@
         <v>1</v>
       </c>
       <c r="K46" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L46" s="12"/>
       <c r="M46" s="10"/>
@@ -3489,30 +3573,30 @@
         <v>4</v>
       </c>
       <c r="O46" s="10" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="29" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B47" s="39" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C47" s="3">
         <v>4.99</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E47" s="11" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F47" s="5">
         <v>45</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="H47" s="5">
         <v>8410123457080</v>
@@ -3522,7 +3606,7 @@
         <v>260</v>
       </c>
       <c r="K47" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L47" s="12"/>
       <c r="M47" s="10"/>
@@ -3532,25 +3616,25 @@
     </row>
     <row r="48" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A48" s="29" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B48" s="39" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C48" s="3">
         <v>5.89</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E48" s="11" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F48" s="5">
         <v>35</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="H48" s="5">
         <v>8410123457097</v>
@@ -3560,11 +3644,11 @@
         <v>350</v>
       </c>
       <c r="K48" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L48" s="12"/>
       <c r="M48" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="N48" s="26">
         <v>10</v>
@@ -3572,25 +3656,25 @@
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="29" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B49" s="39" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C49" s="3">
         <v>2.79</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E49" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F49" s="5">
         <v>65</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="H49" s="5">
         <v>8410123457103</v>
@@ -3600,11 +3684,11 @@
         <v>500</v>
       </c>
       <c r="K49" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L49" s="12"/>
       <c r="M49" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N49" s="26">
         <v>4</v>
@@ -3612,25 +3696,25 @@
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" s="29" t="s">
+        <v>172</v>
+      </c>
+      <c r="B50" s="39" t="s">
         <v>173</v>
-      </c>
-      <c r="B50" s="39" t="s">
-        <v>174</v>
       </c>
       <c r="C50" s="3">
         <v>2.65</v>
       </c>
       <c r="D50" s="11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E50" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F50" s="5">
         <v>40</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="H50" s="5">
         <v>8410123457110</v>
@@ -3640,11 +3724,11 @@
         <v>200</v>
       </c>
       <c r="K50" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L50" s="12"/>
       <c r="M50" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N50" s="26">
         <v>4</v>
@@ -3652,25 +3736,25 @@
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" s="29" t="s">
+        <v>174</v>
+      </c>
+      <c r="B51" s="39" t="s">
         <v>175</v>
-      </c>
-      <c r="B51" s="39" t="s">
-        <v>176</v>
       </c>
       <c r="C51" s="3">
         <v>3.29</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F51" s="5">
         <v>80</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="H51" s="5">
         <v>8410123457127</v>
@@ -3680,11 +3764,11 @@
         <v>300</v>
       </c>
       <c r="K51" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L51" s="12"/>
       <c r="M51" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="N51" s="26">
         <v>4</v>
@@ -3692,25 +3776,25 @@
     </row>
     <row r="52" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="29" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B52" s="39" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C52" s="3">
         <v>1.99</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E52" s="11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F52" s="5">
         <v>60</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="H52" s="5">
         <v>8410123457134</v>
@@ -3720,11 +3804,11 @@
         <v>460</v>
       </c>
       <c r="K52" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L52" s="12"/>
       <c r="M52" s="10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="N52" s="26">
         <v>4</v>
@@ -3732,25 +3816,25 @@
     </row>
     <row r="53" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="29" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B53" s="39" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C53" s="3">
         <v>1.45</v>
       </c>
       <c r="D53" s="11" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E53" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F53" s="5">
         <v>40</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="H53" s="5">
         <v>8410123457141</v>
@@ -3760,11 +3844,11 @@
         <v>1</v>
       </c>
       <c r="K53" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L53" s="12"/>
       <c r="M53" s="10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="N53" s="26">
         <v>4</v>
@@ -3772,25 +3856,25 @@
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="29" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B54" s="39" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C54" s="3">
         <v>2.19</v>
       </c>
       <c r="D54" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E54" s="11" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F54" s="5">
         <v>70</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="H54" s="5">
         <v>8410123457158</v>
@@ -3800,7 +3884,7 @@
         <v>500</v>
       </c>
       <c r="K54" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L54" s="12"/>
       <c r="M54" s="10"/>
@@ -3810,25 +3894,25 @@
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" s="29" t="s">
+        <v>178</v>
+      </c>
+      <c r="B55" s="39" t="s">
         <v>179</v>
-      </c>
-      <c r="B55" s="39" t="s">
-        <v>180</v>
       </c>
       <c r="C55" s="3">
         <v>1.49</v>
       </c>
       <c r="D55" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F55" s="5">
         <v>85</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="H55" s="5">
         <v>8410123457165</v>
@@ -3838,11 +3922,11 @@
         <v>500</v>
       </c>
       <c r="K55" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L55" s="12"/>
       <c r="M55" s="10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="N55" s="26">
         <v>10</v>
@@ -3850,25 +3934,25 @@
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" s="29" t="s">
+        <v>180</v>
+      </c>
+      <c r="B56" s="39" t="s">
         <v>181</v>
-      </c>
-      <c r="B56" s="39" t="s">
-        <v>182</v>
       </c>
       <c r="C56" s="3">
         <v>3.45</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F56" s="5">
         <v>30</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="H56" s="5">
         <v>8410123457172</v>
@@ -3882,7 +3966,7 @@
       </c>
       <c r="L56" s="12"/>
       <c r="M56" s="10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="N56" s="26">
         <v>10</v>
@@ -3890,25 +3974,25 @@
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A57" s="29" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B57" s="39" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C57" s="3">
         <v>1.35</v>
       </c>
       <c r="D57" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F57" s="5">
         <v>90</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="H57" s="5">
         <v>8410123457189</v>
@@ -3918,7 +4002,7 @@
         <v>400</v>
       </c>
       <c r="K57" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L57" s="12"/>
       <c r="M57" s="10"/>
@@ -3928,25 +4012,25 @@
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A58" s="29" t="s">
+        <v>183</v>
+      </c>
+      <c r="B58" s="39" t="s">
         <v>184</v>
-      </c>
-      <c r="B58" s="39" t="s">
-        <v>185</v>
       </c>
       <c r="C58" s="3">
         <v>2.95</v>
       </c>
       <c r="D58" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E58" s="11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F58" s="5">
         <v>25</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="H58" s="5">
         <v>8410123457196</v>
@@ -3960,7 +4044,7 @@
       </c>
       <c r="L58" s="12"/>
       <c r="M58" s="10" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="N58" s="26">
         <v>10</v>
@@ -3968,25 +4052,25 @@
     </row>
     <row r="59" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A59" s="29" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B59" s="39" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C59" s="3">
         <v>3.25</v>
       </c>
       <c r="D59" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E59" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F59" s="5">
         <v>55</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="H59" s="5">
         <v>8410123457202</v>
@@ -3996,11 +4080,11 @@
         <v>550</v>
       </c>
       <c r="K59" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L59" s="12"/>
       <c r="M59" s="25" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="N59" s="26">
         <v>10</v>
@@ -4008,25 +4092,25 @@
     </row>
     <row r="60" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A60" s="29" t="s">
+        <v>189</v>
+      </c>
+      <c r="B60" s="39" t="s">
         <v>190</v>
-      </c>
-      <c r="B60" s="39" t="s">
-        <v>191</v>
       </c>
       <c r="C60" s="3">
         <v>3.29</v>
       </c>
       <c r="D60" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E60" s="11" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F60" s="5">
         <v>60</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="H60" s="5">
         <v>8410123457219</v>
@@ -4036,7 +4120,7 @@
         <v>250</v>
       </c>
       <c r="K60" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L60" s="12"/>
       <c r="M60" s="10"/>
@@ -4046,10 +4130,10 @@
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A61" s="29" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B61" s="39" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="C61" s="3">
         <v>0.75</v>
@@ -4064,7 +4148,7 @@
         <v>100</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="H61" s="5">
         <v>8410123457226</v>
@@ -4074,7 +4158,7 @@
         <v>33</v>
       </c>
       <c r="K61" s="10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="L61" s="12"/>
       <c r="M61" s="10"/>
@@ -4084,10 +4168,10 @@
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A62" s="29" t="s">
+        <v>192</v>
+      </c>
+      <c r="B62" s="39" t="s">
         <v>193</v>
-      </c>
-      <c r="B62" s="39" t="s">
-        <v>194</v>
       </c>
       <c r="C62" s="3">
         <v>0.62</v>
@@ -4102,7 +4186,7 @@
         <v>180</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="H62" s="5">
         <v>8410123457233</v>
@@ -4122,10 +4206,10 @@
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A63" s="29" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B63" s="39" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C63" s="3">
         <v>2.4900000000000002</v>
@@ -4134,13 +4218,13 @@
         <v>22</v>
       </c>
       <c r="E63" s="11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F63" s="5">
         <v>90</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="H63" s="5">
         <v>8410123457240</v>
@@ -4150,7 +4234,7 @@
         <v>130</v>
       </c>
       <c r="K63" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L63" s="12"/>
       <c r="M63" s="10"/>
@@ -4160,25 +4244,25 @@
     </row>
     <row r="64" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A64" s="29" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="B64" s="39" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C64" s="3">
         <v>4.25</v>
       </c>
       <c r="D64" s="11" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E64" s="11" t="s">
-        <v>198</v>
+        <v>321</v>
       </c>
       <c r="F64" s="5">
         <v>55</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="H64" s="5">
         <v>8410123457257</v>
@@ -4188,11 +4272,11 @@
         <v>400</v>
       </c>
       <c r="K64" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L64" s="12"/>
       <c r="M64" s="25" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="N64" s="26">
         <v>10</v>
@@ -4200,25 +4284,25 @@
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="29" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B65" s="39" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C65" s="3">
         <v>2.19</v>
       </c>
       <c r="D65" s="11" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E65" s="11" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F65" s="5">
         <v>70</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="H65" s="5">
         <v>8410123457264</v>
@@ -4228,11 +4312,11 @@
         <v>600</v>
       </c>
       <c r="K65" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L65" s="12"/>
       <c r="M65" s="10" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="N65" s="26">
         <v>10</v>
@@ -4240,25 +4324,25 @@
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="29" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="B66" s="39" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C66" s="3">
         <v>7.5</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E66" s="11" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="F66" s="5">
         <v>14</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="H66" s="5">
         <v>124</v>
@@ -4268,7 +4352,7 @@
         <v>1</v>
       </c>
       <c r="K66" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L66" s="12"/>
       <c r="M66" s="10"/>
@@ -4278,25 +4362,25 @@
     </row>
     <row r="67" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A67" s="29" t="s">
+        <v>303</v>
+      </c>
+      <c r="B67" s="39" t="s">
         <v>305</v>
-      </c>
-      <c r="B67" s="39" t="s">
-        <v>307</v>
       </c>
       <c r="C67" s="3">
         <v>1.2</v>
       </c>
       <c r="D67" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="E67" s="11" t="s">
         <v>158</v>
-      </c>
-      <c r="E67" s="11" t="s">
-        <v>159</v>
       </c>
       <c r="F67" s="5">
         <v>110</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="H67" s="5">
         <v>40111490</v>
@@ -4306,11 +4390,11 @@
         <v>45</v>
       </c>
       <c r="K67" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L67" s="12"/>
       <c r="M67" s="25" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="N67" s="26">
         <v>21</v>
@@ -4318,25 +4402,25 @@
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="29" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="B68" s="39" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C68" s="3">
         <v>0.85</v>
       </c>
       <c r="D68" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="E68" s="11" t="s">
         <v>158</v>
-      </c>
-      <c r="E68" s="11" t="s">
-        <v>159</v>
       </c>
       <c r="F68" s="5">
         <v>120</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="H68" s="5">
         <v>8432750194623</v>
@@ -4346,11 +4430,11 @@
         <v>45</v>
       </c>
       <c r="K68" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L68" s="12"/>
       <c r="M68" s="10" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="N68" s="26">
         <v>10</v>
@@ -4358,25 +4442,25 @@
     </row>
     <row r="69" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A69" s="29" t="s">
+        <v>310</v>
+      </c>
+      <c r="B69" s="39" t="s">
         <v>312</v>
-      </c>
-      <c r="B69" s="39" t="s">
-        <v>314</v>
       </c>
       <c r="C69" s="3">
         <v>2.29</v>
       </c>
       <c r="D69" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E69" s="11" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="F69" s="5">
         <v>65</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="H69" s="5">
         <v>88888</v>
@@ -4386,7 +4470,7 @@
         <v>1</v>
       </c>
       <c r="K69" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L69" s="12"/>
       <c r="M69" s="25"/>
@@ -4394,136 +4478,322 @@
         <v>4</v>
       </c>
       <c r="O69" s="10" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A70" s="29" t="s">
         <v>315</v>
       </c>
-    </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A70" s="29"/>
-      <c r="B70" s="39"/>
-      <c r="C70" s="3"/>
-      <c r="D70" s="11"/>
-      <c r="E70" s="11"/>
-      <c r="F70" s="5"/>
-      <c r="G70" s="1"/>
-      <c r="H70" s="5"/>
+      <c r="B70" s="39" t="s">
+        <v>316</v>
+      </c>
+      <c r="C70" s="3">
+        <v>1.61</v>
+      </c>
+      <c r="D70" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="E70" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="F70" s="5">
+        <v>100</v>
+      </c>
+      <c r="G70" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="H70" s="5">
+        <v>8410066070060</v>
+      </c>
       <c r="I70" s="12"/>
-      <c r="J70" s="9"/>
-      <c r="K70" s="10"/>
+      <c r="J70" s="9">
+        <v>300</v>
+      </c>
+      <c r="K70" s="10" t="s">
+        <v>38</v>
+      </c>
       <c r="L70" s="12"/>
       <c r="M70" s="25"/>
-      <c r="N70" s="26"/>
-    </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A71" s="29"/>
-      <c r="B71" s="39"/>
-      <c r="C71" s="3"/>
-      <c r="D71" s="11"/>
-      <c r="E71" s="11"/>
-      <c r="F71" s="5"/>
-      <c r="G71" s="1"/>
-      <c r="H71" s="5"/>
+      <c r="N70" s="26">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="71" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A71" s="29" t="s">
+        <v>322</v>
+      </c>
+      <c r="B71" s="39" t="s">
+        <v>323</v>
+      </c>
+      <c r="C71" s="3">
+        <v>0.99</v>
+      </c>
+      <c r="D71" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E71" s="11" t="s">
+        <v>317</v>
+      </c>
+      <c r="F71" s="5">
+        <v>100</v>
+      </c>
+      <c r="G71" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="H71" s="5">
+        <v>8410569310014</v>
+      </c>
       <c r="I71" s="12"/>
-      <c r="J71" s="9"/>
-      <c r="K71" s="10"/>
+      <c r="J71" s="9">
+        <v>33</v>
+      </c>
+      <c r="K71" s="10" t="s">
+        <v>29</v>
+      </c>
       <c r="L71" s="12"/>
-      <c r="M71" s="25"/>
-      <c r="N71" s="26"/>
+      <c r="M71" s="25" t="s">
+        <v>110</v>
+      </c>
+      <c r="N71" s="26">
+        <v>10</v>
+      </c>
     </row>
     <row r="72" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A72" s="29"/>
-      <c r="B72" s="39"/>
-      <c r="C72" s="3"/>
-      <c r="D72" s="11"/>
-      <c r="E72" s="11"/>
-      <c r="F72" s="5"/>
-      <c r="G72" s="1"/>
-      <c r="H72" s="5"/>
+      <c r="A72" s="29" t="s">
+        <v>318</v>
+      </c>
+      <c r="B72" s="39" t="s">
+        <v>319</v>
+      </c>
+      <c r="C72" s="3">
+        <v>1.08</v>
+      </c>
+      <c r="D72" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E72" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F72" s="5">
+        <v>150</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="H72" s="5">
+        <v>5449000322388</v>
+      </c>
       <c r="I72" s="12"/>
-      <c r="J72" s="9"/>
-      <c r="K72" s="10"/>
+      <c r="J72" s="9">
+        <v>33</v>
+      </c>
+      <c r="K72" s="10" t="s">
+        <v>29</v>
+      </c>
       <c r="L72" s="12"/>
       <c r="M72" s="25"/>
-      <c r="N72" s="26"/>
+      <c r="N72" s="26">
+        <v>21</v>
+      </c>
     </row>
     <row r="73" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A73" s="29"/>
-      <c r="B73" s="39"/>
-      <c r="C73" s="3"/>
-      <c r="D73" s="11"/>
-      <c r="E73" s="11"/>
-      <c r="F73" s="5"/>
-      <c r="G73" s="1"/>
-      <c r="H73" s="5"/>
+      <c r="A73" s="29" t="s">
+        <v>330</v>
+      </c>
+      <c r="B73" s="39" t="s">
+        <v>333</v>
+      </c>
+      <c r="C73" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="D73" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E73" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="F73" s="5">
+        <v>80</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="H73" s="5">
+        <v>8402001024900</v>
+      </c>
       <c r="I73" s="12"/>
-      <c r="J73" s="9"/>
-      <c r="K73" s="10"/>
+      <c r="J73" s="9">
+        <v>6</v>
+      </c>
+      <c r="K73" s="10" t="s">
+        <v>331</v>
+      </c>
       <c r="L73" s="12"/>
-      <c r="M73" s="25"/>
-      <c r="N73" s="26"/>
-    </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A74" s="29"/>
-      <c r="B74" s="39"/>
-      <c r="C74" s="3"/>
-      <c r="D74" s="11"/>
-      <c r="E74" s="11"/>
-      <c r="F74" s="5"/>
-      <c r="G74" s="1"/>
-      <c r="H74" s="5"/>
+      <c r="M73" s="25" t="s">
+        <v>48</v>
+      </c>
+      <c r="N73" s="26">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="74" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+      <c r="A74" s="29" t="s">
+        <v>320</v>
+      </c>
+      <c r="B74" s="39" t="s">
+        <v>335</v>
+      </c>
+      <c r="C74" s="3">
+        <v>1.35</v>
+      </c>
+      <c r="D74" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="E74" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="F74" s="5">
+        <v>60</v>
+      </c>
+      <c r="G74" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="H74" s="5">
+        <v>8410173001018</v>
+      </c>
       <c r="I74" s="12"/>
-      <c r="J74" s="9"/>
-      <c r="K74" s="10"/>
+      <c r="J74" s="9">
+        <v>125</v>
+      </c>
+      <c r="K74" s="10" t="s">
+        <v>38</v>
+      </c>
       <c r="L74" s="12"/>
-      <c r="M74" s="25"/>
-      <c r="N74" s="26"/>
+      <c r="M74" s="25" t="s">
+        <v>332</v>
+      </c>
+      <c r="N74" s="26">
+        <v>10</v>
+      </c>
     </row>
     <row r="75" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A75" s="29"/>
-      <c r="B75" s="39"/>
-      <c r="C75" s="3"/>
-      <c r="D75" s="11"/>
-      <c r="E75" s="11"/>
-      <c r="F75" s="5"/>
-      <c r="G75" s="1"/>
-      <c r="H75" s="5"/>
-      <c r="I75" s="12"/>
-      <c r="J75" s="9"/>
-      <c r="K75" s="10"/>
+      <c r="A75" s="29" t="s">
+        <v>324</v>
+      </c>
+      <c r="B75" s="39" t="s">
+        <v>325</v>
+      </c>
+      <c r="C75" s="3">
+        <v>0.8</v>
+      </c>
+      <c r="D75" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E75" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F75" s="5">
+        <v>150</v>
+      </c>
+      <c r="G75" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="H75" s="5">
+        <v>5449000120960</v>
+      </c>
+      <c r="I75" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="J75" s="9">
+        <v>33</v>
+      </c>
+      <c r="K75" s="10" t="s">
+        <v>29</v>
+      </c>
       <c r="L75" s="12"/>
       <c r="M75" s="25"/>
-      <c r="N75" s="26"/>
+      <c r="N75" s="26">
+        <v>21</v>
+      </c>
     </row>
     <row r="76" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A76" s="29"/>
-      <c r="B76" s="39"/>
-      <c r="C76" s="3"/>
-      <c r="D76" s="11"/>
-      <c r="E76" s="11"/>
-      <c r="F76" s="5"/>
-      <c r="G76" s="1"/>
-      <c r="H76" s="5"/>
+      <c r="A76" s="29" t="s">
+        <v>341</v>
+      </c>
+      <c r="B76" s="39" t="s">
+        <v>342</v>
+      </c>
+      <c r="C76" s="3">
+        <v>11.95</v>
+      </c>
+      <c r="D76" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="E76" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="F76" s="5">
+        <v>0</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="H76" s="5">
+        <v>8410066001002</v>
+      </c>
       <c r="I76" s="12"/>
-      <c r="J76" s="9"/>
-      <c r="K76" s="10"/>
+      <c r="J76" s="9">
+        <v>5</v>
+      </c>
+      <c r="K76" s="10" t="s">
+        <v>28</v>
+      </c>
       <c r="L76" s="12"/>
       <c r="M76" s="25"/>
-      <c r="N76" s="26"/>
+      <c r="N76" s="26">
+        <v>10</v>
+      </c>
     </row>
     <row r="77" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A77" s="29"/>
-      <c r="B77" s="39"/>
-      <c r="C77" s="3"/>
-      <c r="D77" s="11"/>
-      <c r="E77" s="11"/>
-      <c r="F77" s="5"/>
-      <c r="G77" s="1"/>
-      <c r="H77" s="5"/>
+      <c r="A77" s="29" t="s">
+        <v>343</v>
+      </c>
+      <c r="B77" s="39" t="s">
+        <v>337</v>
+      </c>
+      <c r="C77" s="3">
+        <v>3.29</v>
+      </c>
+      <c r="D77" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="E77" s="11" t="s">
+        <v>338</v>
+      </c>
+      <c r="F77" s="5">
+        <v>50</v>
+      </c>
+      <c r="G77" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="H77" s="5">
+        <v>8410343001234</v>
+      </c>
       <c r="I77" s="12"/>
-      <c r="J77" s="9"/>
-      <c r="K77" s="10"/>
+      <c r="J77" s="9">
+        <v>200</v>
+      </c>
+      <c r="K77" s="10" t="s">
+        <v>38</v>
+      </c>
       <c r="L77" s="12"/>
-      <c r="M77" s="25"/>
-      <c r="N77" s="26"/>
+      <c r="M77" s="25" t="s">
+        <v>339</v>
+      </c>
+      <c r="N77" s="26">
+        <v>10</v>
+      </c>
     </row>
     <row r="78" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A78" s="29"/>
@@ -4566,7 +4836,7 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="22" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B1" s="22" t="s">
         <v>0</v>
@@ -4575,42 +4845,42 @@
         <v>1</v>
       </c>
       <c r="D1" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="E1" s="22" t="s">
+      <c r="F1" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="F1" s="22" t="s">
-        <v>55</v>
-      </c>
-      <c r="G1" s="22" t="s">
+      <c r="H1" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="H1" s="22" t="s">
+      <c r="I1" s="22" t="s">
         <v>60</v>
-      </c>
-      <c r="I1" s="22" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D2" s="17" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="F2" s="20" t="s">
         <v>63</v>
-      </c>
-      <c r="F2" s="20" t="s">
-        <v>64</v>
       </c>
       <c r="G2" s="18">
         <v>46082</v>
@@ -4624,22 +4894,22 @@
     </row>
     <row r="3" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D3" s="17" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F3" s="20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G3" s="18">
         <v>46082</v>
@@ -4653,22 +4923,22 @@
     </row>
     <row r="4" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="B4" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="B4" s="15" t="s">
-        <v>70</v>
-      </c>
       <c r="C4" s="16" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D4" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="E4" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="F4" s="20" t="s">
         <v>73</v>
-      </c>
-      <c r="E4" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="F4" s="20" t="s">
-        <v>74</v>
       </c>
       <c r="G4" s="18">
         <v>46082</v>
@@ -4682,22 +4952,22 @@
     </row>
     <row r="5" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="20" t="s">
+        <v>75</v>
+      </c>
+      <c r="B5" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="B5" s="16" t="s">
-        <v>77</v>
-      </c>
       <c r="C5" s="16" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G5" s="23">
         <v>46082</v>

</xml_diff>